<commit_message>
Publish Tacen_2022_WC, Vaires_2023_WC, Tacen_2018_WC
</commit_message>
<xml_diff>
--- a/events/Tacen_2018_WC/Tacen_2018_WC_start.xlsx
+++ b/events/Tacen_2018_WC/Tacen_2018_WC_start.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W368"/>
+  <dimension ref="A1:AC368"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -519,17 +519,47 @@
       </c>
       <c r="U1" t="inlineStr">
         <is>
+          <t>Name4</t>
+        </is>
+      </c>
+      <c r="V1" t="inlineStr">
+        <is>
+          <t>Name5</t>
+        </is>
+      </c>
+      <c r="W1" t="inlineStr">
+        <is>
+          <t>Name6</t>
+        </is>
+      </c>
+      <c r="X1" t="inlineStr">
+        <is>
           <t>ICF_ID1</t>
         </is>
       </c>
-      <c r="V1" t="inlineStr">
+      <c r="Y1" t="inlineStr">
         <is>
           <t>ICF_ID2</t>
         </is>
       </c>
-      <c r="W1" t="inlineStr">
+      <c r="Z1" t="inlineStr">
         <is>
           <t>ICF_ID3</t>
+        </is>
+      </c>
+      <c r="AA1" t="inlineStr">
+        <is>
+          <t>ICF_ID4</t>
+        </is>
+      </c>
+      <c r="AB1" t="inlineStr">
+        <is>
+          <t>ICF_ID5</t>
+        </is>
+      </c>
+      <c r="AC1" t="inlineStr">
+        <is>
+          <t>ICF_ID6</t>
         </is>
       </c>
     </row>
@@ -1128,7 +1158,7 @@
           <t>MOORHOUSE Eoin</t>
         </is>
       </c>
-      <c r="U13" t="inlineStr">
+      <c r="X13" t="inlineStr">
         <is>
           <t>70052</t>
         </is>
@@ -1186,7 +1216,7 @@
           <t>TANIGUCHI Kazuya</t>
         </is>
       </c>
-      <c r="U14" t="inlineStr">
+      <c r="X14" t="inlineStr">
         <is>
           <t>39699</t>
         </is>
@@ -1244,7 +1274,7 @@
           <t>HODSON Ethan</t>
         </is>
       </c>
-      <c r="U15" t="inlineStr">
+      <c r="X15" t="inlineStr">
         <is>
           <t>38437</t>
         </is>
@@ -1302,7 +1332,7 @@
           <t>GESTIN Nicolas</t>
         </is>
       </c>
-      <c r="U16" t="inlineStr">
+      <c r="X16" t="inlineStr">
         <is>
           <t>71961</t>
         </is>
@@ -1360,7 +1390,7 @@
           <t>MICOZZI Flavio</t>
         </is>
       </c>
-      <c r="U17" t="inlineStr">
+      <c r="X17" t="inlineStr">
         <is>
           <t>77363</t>
         </is>
@@ -1524,7 +1554,7 @@
           <t>ABBOTT Thomas</t>
         </is>
       </c>
-      <c r="U20" t="inlineStr">
+      <c r="X20" t="inlineStr">
         <is>
           <t>36514</t>
         </is>
@@ -1582,7 +1612,7 @@
           <t>BOURHIS Yves</t>
         </is>
       </c>
-      <c r="U21" t="inlineStr">
+      <c r="X21" t="inlineStr">
         <is>
           <t>63237</t>
         </is>
@@ -1640,7 +1670,7 @@
           <t>CHIARELLO Gelindo</t>
         </is>
       </c>
-      <c r="U22" t="inlineStr">
+      <c r="X22" t="inlineStr">
         <is>
           <t>39956</t>
         </is>
@@ -1698,7 +1728,7 @@
           <t>LOWTHER Steven</t>
         </is>
       </c>
-      <c r="U23" t="inlineStr">
+      <c r="X23" t="inlineStr">
         <is>
           <t>44811</t>
         </is>
@@ -1756,7 +1786,7 @@
           <t>SASAKI Shota</t>
         </is>
       </c>
-      <c r="U24" t="inlineStr">
+      <c r="X24" t="inlineStr">
         <is>
           <t>41610</t>
         </is>
@@ -1814,7 +1844,7 @@
           <t>SZTUBA Igor</t>
         </is>
       </c>
-      <c r="U25" t="inlineStr">
+      <c r="X25" t="inlineStr">
         <is>
           <t>35087</t>
         </is>
@@ -1872,7 +1902,7 @@
           <t>CECCON Paolo</t>
         </is>
       </c>
-      <c r="U26" t="inlineStr">
+      <c r="X26" t="inlineStr">
         <is>
           <t>39903</t>
         </is>
@@ -1930,7 +1960,7 @@
           <t>TRUMMER Timo</t>
         </is>
       </c>
-      <c r="U27" t="inlineStr">
+      <c r="X27" t="inlineStr">
         <is>
           <t>41599</t>
         </is>
@@ -1988,7 +2018,7 @@
           <t>SZTUBA Kacper</t>
         </is>
       </c>
-      <c r="U28" t="inlineStr">
+      <c r="X28" t="inlineStr">
         <is>
           <t>53636</t>
         </is>
@@ -2046,7 +2076,7 @@
           <t>MARINIC Matija</t>
         </is>
       </c>
-      <c r="U29" t="inlineStr">
+      <c r="X29" t="inlineStr">
         <is>
           <t>35595</t>
         </is>
@@ -2104,7 +2134,7 @@
           <t>LOKKEN Zachary</t>
         </is>
       </c>
-      <c r="U30" t="inlineStr">
+      <c r="X30" t="inlineStr">
         <is>
           <t>35069</t>
         </is>
@@ -2162,7 +2192,7 @@
           <t>JANE Michal</t>
         </is>
       </c>
-      <c r="U31" t="inlineStr">
+      <c r="X31" t="inlineStr">
         <is>
           <t>35059</t>
         </is>
@@ -2220,7 +2250,7 @@
           <t>LENARCIC Jure</t>
         </is>
       </c>
-      <c r="U32" t="inlineStr">
+      <c r="X32" t="inlineStr">
         <is>
           <t>36259</t>
         </is>
@@ -2278,7 +2308,7 @@
           <t>RAK Tomas</t>
         </is>
       </c>
-      <c r="U33" t="inlineStr">
+      <c r="X33" t="inlineStr">
         <is>
           <t>35056</t>
         </is>
@@ -2336,7 +2366,7 @@
           <t>JOLY Cedric</t>
         </is>
       </c>
-      <c r="U34" t="inlineStr">
+      <c r="X34" t="inlineStr">
         <is>
           <t>35681</t>
         </is>
@@ -2394,7 +2424,7 @@
           <t>TILLARD Pierre-Antoine</t>
         </is>
       </c>
-      <c r="U35" t="inlineStr">
+      <c r="X35" t="inlineStr">
         <is>
           <t>35413</t>
         </is>
@@ -2452,7 +2482,7 @@
           <t>BERCIC Anze</t>
         </is>
       </c>
-      <c r="U36" t="inlineStr">
+      <c r="X36" t="inlineStr">
         <is>
           <t>36253</t>
         </is>
@@ -2510,7 +2540,7 @@
           <t>HANEDA Takuya</t>
         </is>
       </c>
-      <c r="U37" t="inlineStr">
+      <c r="X37" t="inlineStr">
         <is>
           <t>36481</t>
         </is>
@@ -2568,7 +2598,7 @@
           <t>MIRGORODSKY Marko</t>
         </is>
       </c>
-      <c r="U38" t="inlineStr">
+      <c r="X38" t="inlineStr">
         <is>
           <t>42019</t>
         </is>
@@ -2626,7 +2656,7 @@
           <t>EICHFELD Casey</t>
         </is>
       </c>
-      <c r="U39" t="inlineStr">
+      <c r="X39" t="inlineStr">
         <is>
           <t>35067</t>
         </is>
@@ -2684,7 +2714,7 @@
           <t>HEDWIG Grzegorz</t>
         </is>
       </c>
-      <c r="U40" t="inlineStr">
+      <c r="X40" t="inlineStr">
         <is>
           <t>35465</t>
         </is>
@@ -2742,7 +2772,7 @@
           <t>ROHAN Lukas</t>
         </is>
       </c>
-      <c r="U41" t="inlineStr">
+      <c r="X41" t="inlineStr">
         <is>
           <t>36114</t>
         </is>
@@ -2800,7 +2830,7 @@
           <t>ANTON Franz</t>
         </is>
       </c>
-      <c r="U42" t="inlineStr">
+      <c r="X42" t="inlineStr">
         <is>
           <t>35137</t>
         </is>
@@ -2858,7 +2888,7 @@
           <t>BOZIC Luka</t>
         </is>
       </c>
-      <c r="U43" t="inlineStr">
+      <c r="X43" t="inlineStr">
         <is>
           <t>36269</t>
         </is>
@@ -2916,7 +2946,7 @@
           <t>GARGAUD CHANUT Denis</t>
         </is>
       </c>
-      <c r="U44" t="inlineStr">
+      <c r="X44" t="inlineStr">
         <is>
           <t>35177</t>
         </is>
@@ -2974,7 +3004,7 @@
           <t>MARTIKAN Michal</t>
         </is>
       </c>
-      <c r="U45" t="inlineStr">
+      <c r="X45" t="inlineStr">
         <is>
           <t>35365</t>
         </is>
@@ -3032,7 +3062,7 @@
           <t>BENUS Matej</t>
         </is>
       </c>
-      <c r="U46" t="inlineStr">
+      <c r="X46" t="inlineStr">
         <is>
           <t>35353</t>
         </is>
@@ -3090,7 +3120,7 @@
           <t>SLAFKOVSKY Alexander</t>
         </is>
       </c>
-      <c r="U47" t="inlineStr">
+      <c r="X47" t="inlineStr">
         <is>
           <t>35129</t>
         </is>
@@ -3148,7 +3178,7 @@
           <t>SAVSEK Benjamin</t>
         </is>
       </c>
-      <c r="U48" t="inlineStr">
+      <c r="X48" t="inlineStr">
         <is>
           <t>36218</t>
         </is>
@@ -3206,7 +3236,7 @@
           <t>TASIADIS Sideris</t>
         </is>
       </c>
-      <c r="U49" t="inlineStr">
+      <c r="X49" t="inlineStr">
         <is>
           <t>35135</t>
         </is>
@@ -3264,7 +3294,7 @@
           <t>LEAVER Lois</t>
         </is>
       </c>
-      <c r="U50" t="inlineStr">
+      <c r="X50" t="inlineStr">
         <is>
           <t>83842</t>
         </is>
@@ -3322,7 +3352,7 @@
           <t>BENGERI Katja</t>
         </is>
       </c>
-      <c r="U51" t="inlineStr">
+      <c r="X51" t="inlineStr">
         <is>
           <t>72852</t>
         </is>
@@ -3380,7 +3410,7 @@
           <t>OGILVIE Sophie</t>
         </is>
       </c>
-      <c r="U52" t="inlineStr">
+      <c r="X52" t="inlineStr">
         <is>
           <t>53134</t>
         </is>
@@ -3438,7 +3468,7 @@
           <t>DELASSUS Marjorie</t>
         </is>
       </c>
-      <c r="U53" t="inlineStr">
+      <c r="X53" t="inlineStr">
         <is>
           <t>71964</t>
         </is>
@@ -3496,7 +3526,7 @@
           <t>RIHOVA Eva</t>
         </is>
       </c>
-      <c r="U54" t="inlineStr">
+      <c r="X54" t="inlineStr">
         <is>
           <t>51791</t>
         </is>
@@ -3554,7 +3584,7 @@
           <t>FABER Anna</t>
         </is>
       </c>
-      <c r="U55" t="inlineStr">
+      <c r="X55" t="inlineStr">
         <is>
           <t>39059</t>
         </is>
@@ -3612,7 +3642,7 @@
           <t>MARX Alena</t>
         </is>
       </c>
-      <c r="U56" t="inlineStr">
+      <c r="X56" t="inlineStr">
         <is>
           <t>68844</t>
         </is>
@@ -3670,7 +3700,7 @@
           <t>MISHIMA Ren</t>
         </is>
       </c>
-      <c r="U57" t="inlineStr">
+      <c r="X57" t="inlineStr">
         <is>
           <t>37757</t>
         </is>
@@ -3728,7 +3758,7 @@
           <t>MURZOVA Lucia</t>
         </is>
       </c>
-      <c r="U58" t="inlineStr">
+      <c r="X58" t="inlineStr">
         <is>
           <t>60316</t>
         </is>
@@ -3786,7 +3816,7 @@
           <t>SRIBAR Ria</t>
         </is>
       </c>
-      <c r="U59" t="inlineStr">
+      <c r="X59" t="inlineStr">
         <is>
           <t>75645</t>
         </is>
@@ -3844,7 +3874,7 @@
           <t>DONNELLY Sage</t>
         </is>
       </c>
-      <c r="U60" t="inlineStr">
+      <c r="X60" t="inlineStr">
         <is>
           <t>60119</t>
         </is>
@@ -3902,7 +3932,7 @@
           <t>MITASIKOVA Monika</t>
         </is>
       </c>
-      <c r="U61" t="inlineStr">
+      <c r="X61" t="inlineStr">
         <is>
           <t>75445</t>
         </is>
@@ -3960,7 +3990,7 @@
           <t>LUCATO Eleonora</t>
         </is>
       </c>
-      <c r="U62" t="inlineStr">
+      <c r="X62" t="inlineStr">
         <is>
           <t>35222</t>
         </is>
@@ -4018,7 +4048,7 @@
           <t>HAMER-EVANS Megan</t>
         </is>
       </c>
-      <c r="U63" t="inlineStr">
+      <c r="X63" t="inlineStr">
         <is>
           <t>55138</t>
         </is>
@@ -4076,7 +4106,7 @@
           <t>MASLEN Amber</t>
         </is>
       </c>
-      <c r="U64" t="inlineStr">
+      <c r="X64" t="inlineStr">
         <is>
           <t>53074</t>
         </is>
@@ -4134,7 +4164,7 @@
           <t>STANOVSKA Sona</t>
         </is>
       </c>
-      <c r="U65" t="inlineStr">
+      <c r="X65" t="inlineStr">
         <is>
           <t>51647</t>
         </is>
@@ -4192,7 +4222,7 @@
           <t>TAKESHITA Yuriko</t>
         </is>
       </c>
-      <c r="U66" t="inlineStr">
+      <c r="X66" t="inlineStr">
         <is>
           <t>36487</t>
         </is>
@@ -4250,7 +4280,7 @@
           <t>OSCHMAUTZ Antonia</t>
         </is>
       </c>
-      <c r="U67" t="inlineStr">
+      <c r="X67" t="inlineStr">
         <is>
           <t>68839</t>
         </is>
@@ -4308,7 +4338,7 @@
           <t>NEE Ashley</t>
         </is>
       </c>
-      <c r="U68" t="inlineStr">
+      <c r="X68" t="inlineStr">
         <is>
           <t>36363</t>
         </is>
@@ -4366,7 +4396,7 @@
           <t>YAZAWA Aki</t>
         </is>
       </c>
-      <c r="U69" t="inlineStr">
+      <c r="X69" t="inlineStr">
         <is>
           <t>36486</t>
         </is>
@@ -4424,7 +4454,7 @@
           <t>NOVAK Ajda</t>
         </is>
       </c>
-      <c r="U70" t="inlineStr">
+      <c r="X70" t="inlineStr">
         <is>
           <t>39079</t>
         </is>
@@ -4482,7 +4512,7 @@
           <t>NEVARILOVA Kristina</t>
         </is>
       </c>
-      <c r="U71" t="inlineStr">
+      <c r="X71" t="inlineStr">
         <is>
           <t>35467</t>
         </is>
@@ -4540,7 +4570,7 @@
           <t>US Viktoriia</t>
         </is>
       </c>
-      <c r="U72" t="inlineStr">
+      <c r="X72" t="inlineStr">
         <is>
           <t>35528</t>
         </is>
@@ -4598,7 +4628,7 @@
           <t>HILGERTOVA Amalie</t>
         </is>
       </c>
-      <c r="U73" t="inlineStr">
+      <c r="X73" t="inlineStr">
         <is>
           <t>36113</t>
         </is>
@@ -4656,7 +4686,7 @@
           <t>WEGMAN Martina</t>
         </is>
       </c>
-      <c r="U74" t="inlineStr">
+      <c r="X74" t="inlineStr">
         <is>
           <t>35345</t>
         </is>
@@ -4714,7 +4744,7 @@
           <t>VOJTOVA Veronika</t>
         </is>
       </c>
-      <c r="U75" t="inlineStr">
+      <c r="X75" t="inlineStr">
         <is>
           <t>35945</t>
         </is>
@@ -4772,7 +4802,7 @@
           <t>LAFONT Marie-Zelia</t>
         </is>
       </c>
-      <c r="U76" t="inlineStr">
+      <c r="X76" t="inlineStr">
         <is>
           <t>35374</t>
         </is>
@@ -4830,7 +4860,7 @@
           <t>LEITNER Lisa</t>
         </is>
       </c>
-      <c r="U77" t="inlineStr">
+      <c r="X77" t="inlineStr">
         <is>
           <t>35305</t>
         </is>
@@ -4888,7 +4918,7 @@
           <t>LAWRENCE Rosalyn</t>
         </is>
       </c>
-      <c r="U78" t="inlineStr">
+      <c r="X78" t="inlineStr">
         <is>
           <t>36531</t>
         </is>
@@ -4946,7 +4976,7 @@
           <t>WOLFFHARDT Viktoria</t>
         </is>
       </c>
-      <c r="U79" t="inlineStr">
+      <c r="X79" t="inlineStr">
         <is>
           <t>35303</t>
         </is>
@@ -5004,7 +5034,7 @@
           <t>PRIGENT Camille</t>
         </is>
       </c>
-      <c r="U80" t="inlineStr">
+      <c r="X80" t="inlineStr">
         <is>
           <t>41566</t>
         </is>
@@ -5062,7 +5092,7 @@
           <t>ZWOLINSKA Klaudia</t>
         </is>
       </c>
-      <c r="U81" t="inlineStr">
+      <c r="X81" t="inlineStr">
         <is>
           <t>42027</t>
         </is>
@@ -5120,7 +5150,7 @@
           <t>KUDEJOVA Katerina</t>
         </is>
       </c>
-      <c r="U82" t="inlineStr">
+      <c r="X82" t="inlineStr">
         <is>
           <t>35034</t>
         </is>
@@ -5178,7 +5208,7 @@
           <t>SCHORNBERG Jasmin</t>
         </is>
       </c>
-      <c r="U83" t="inlineStr">
+      <c r="X83" t="inlineStr">
         <is>
           <t>35206</t>
         </is>
@@ -5236,7 +5266,7 @@
           <t>KRAGELJ Ursa</t>
         </is>
       </c>
-      <c r="U84" t="inlineStr">
+      <c r="X84" t="inlineStr">
         <is>
           <t>36264</t>
         </is>
@@ -5294,7 +5324,7 @@
           <t>HORN Stefanie</t>
         </is>
       </c>
-      <c r="U85" t="inlineStr">
+      <c r="X85" t="inlineStr">
         <is>
           <t>38417</t>
         </is>
@@ -5352,7 +5382,7 @@
           <t>TERCELJ Eva</t>
         </is>
       </c>
-      <c r="U86" t="inlineStr">
+      <c r="X86" t="inlineStr">
         <is>
           <t>36263</t>
         </is>
@@ -5410,7 +5440,7 @@
           <t>KUHNLE Corinna</t>
         </is>
       </c>
-      <c r="U87" t="inlineStr">
+      <c r="X87" t="inlineStr">
         <is>
           <t>35282</t>
         </is>
@@ -5468,7 +5498,7 @@
           <t>FUNK Ricarda</t>
         </is>
       </c>
-      <c r="U88" t="inlineStr">
+      <c r="X88" t="inlineStr">
         <is>
           <t>35122</t>
         </is>
@@ -5526,7 +5556,7 @@
           <t>FOX Jessica</t>
         </is>
       </c>
-      <c r="U89" t="inlineStr">
+      <c r="X89" t="inlineStr">
         <is>
           <t>36526</t>
         </is>
@@ -5584,7 +5614,7 @@
           <t>MOORHOUSE Eoin</t>
         </is>
       </c>
-      <c r="U90" t="inlineStr">
+      <c r="X90" t="inlineStr">
         <is>
           <t>70052</t>
         </is>
@@ -5642,7 +5672,7 @@
           <t>TANIGUCHI Kazuya</t>
         </is>
       </c>
-      <c r="U91" t="inlineStr">
+      <c r="X91" t="inlineStr">
         <is>
           <t>39699</t>
         </is>
@@ -5700,7 +5730,7 @@
           <t>HODSON Ethan</t>
         </is>
       </c>
-      <c r="U92" t="inlineStr">
+      <c r="X92" t="inlineStr">
         <is>
           <t>38437</t>
         </is>
@@ -5758,7 +5788,7 @@
           <t>MICOZZI Flavio</t>
         </is>
       </c>
-      <c r="U93" t="inlineStr">
+      <c r="X93" t="inlineStr">
         <is>
           <t>77363</t>
         </is>
@@ -5869,7 +5899,7 @@
           <t>ABBOTT Thomas</t>
         </is>
       </c>
-      <c r="U95" t="inlineStr">
+      <c r="X95" t="inlineStr">
         <is>
           <t>36514</t>
         </is>
@@ -5927,7 +5957,7 @@
           <t>CHIARELLO Gelindo</t>
         </is>
       </c>
-      <c r="U96" t="inlineStr">
+      <c r="X96" t="inlineStr">
         <is>
           <t>39956</t>
         </is>
@@ -5985,7 +6015,7 @@
           <t>LOWTHER Steven</t>
         </is>
       </c>
-      <c r="U97" t="inlineStr">
+      <c r="X97" t="inlineStr">
         <is>
           <t>44811</t>
         </is>
@@ -6043,7 +6073,7 @@
           <t>SASAKI Shota</t>
         </is>
       </c>
-      <c r="U98" t="inlineStr">
+      <c r="X98" t="inlineStr">
         <is>
           <t>41610</t>
         </is>
@@ -6101,7 +6131,7 @@
           <t>CECCON Paolo</t>
         </is>
       </c>
-      <c r="U99" t="inlineStr">
+      <c r="X99" t="inlineStr">
         <is>
           <t>39903</t>
         </is>
@@ -6159,7 +6189,7 @@
           <t>TRUMMER Timo</t>
         </is>
       </c>
-      <c r="U100" t="inlineStr">
+      <c r="X100" t="inlineStr">
         <is>
           <t>41599</t>
         </is>
@@ -6217,7 +6247,7 @@
           <t>MARINIC Matija</t>
         </is>
       </c>
-      <c r="U101" t="inlineStr">
+      <c r="X101" t="inlineStr">
         <is>
           <t>35595</t>
         </is>
@@ -6275,7 +6305,7 @@
           <t>LOKKEN Zachary</t>
         </is>
       </c>
-      <c r="U102" t="inlineStr">
+      <c r="X102" t="inlineStr">
         <is>
           <t>35069</t>
         </is>
@@ -6333,7 +6363,7 @@
           <t>JANE Michal</t>
         </is>
       </c>
-      <c r="U103" t="inlineStr">
+      <c r="X103" t="inlineStr">
         <is>
           <t>35059</t>
         </is>
@@ -6391,7 +6421,7 @@
           <t>RAK Tomas</t>
         </is>
       </c>
-      <c r="U104" t="inlineStr">
+      <c r="X104" t="inlineStr">
         <is>
           <t>35056</t>
         </is>
@@ -6449,7 +6479,7 @@
           <t>HANEDA Takuya</t>
         </is>
       </c>
-      <c r="U105" t="inlineStr">
+      <c r="X105" t="inlineStr">
         <is>
           <t>36481</t>
         </is>
@@ -6507,7 +6537,7 @@
           <t>GARGAUD CHANUT Denis</t>
         </is>
       </c>
-      <c r="U106" t="inlineStr">
+      <c r="X106" t="inlineStr">
         <is>
           <t>35177</t>
         </is>
@@ -6565,7 +6595,7 @@
           <t>LEAVER Lois</t>
         </is>
       </c>
-      <c r="U107" t="inlineStr">
+      <c r="X107" t="inlineStr">
         <is>
           <t>83842</t>
         </is>
@@ -6623,7 +6653,7 @@
           <t>OGILVIE Sophie</t>
         </is>
       </c>
-      <c r="U108" t="inlineStr">
+      <c r="X108" t="inlineStr">
         <is>
           <t>53134</t>
         </is>
@@ -6681,7 +6711,7 @@
           <t>DELASSUS Marjorie</t>
         </is>
       </c>
-      <c r="U109" t="inlineStr">
+      <c r="X109" t="inlineStr">
         <is>
           <t>71964</t>
         </is>
@@ -6739,7 +6769,7 @@
           <t>RIHOVA Eva</t>
         </is>
       </c>
-      <c r="U110" t="inlineStr">
+      <c r="X110" t="inlineStr">
         <is>
           <t>51791</t>
         </is>
@@ -6797,7 +6827,7 @@
           <t>MARX Alena</t>
         </is>
       </c>
-      <c r="U111" t="inlineStr">
+      <c r="X111" t="inlineStr">
         <is>
           <t>68844</t>
         </is>
@@ -6855,7 +6885,7 @@
           <t>MISHIMA Ren</t>
         </is>
       </c>
-      <c r="U112" t="inlineStr">
+      <c r="X112" t="inlineStr">
         <is>
           <t>37757</t>
         </is>
@@ -6913,7 +6943,7 @@
           <t>MURZOVA Lucia</t>
         </is>
       </c>
-      <c r="U113" t="inlineStr">
+      <c r="X113" t="inlineStr">
         <is>
           <t>60316</t>
         </is>
@@ -6971,7 +7001,7 @@
           <t>SRIBAR Ria</t>
         </is>
       </c>
-      <c r="U114" t="inlineStr">
+      <c r="X114" t="inlineStr">
         <is>
           <t>75645</t>
         </is>
@@ -7029,7 +7059,7 @@
           <t>DONNELLY Sage</t>
         </is>
       </c>
-      <c r="U115" t="inlineStr">
+      <c r="X115" t="inlineStr">
         <is>
           <t>60119</t>
         </is>
@@ -7087,7 +7117,7 @@
           <t>MITASIKOVA Monika</t>
         </is>
       </c>
-      <c r="U116" t="inlineStr">
+      <c r="X116" t="inlineStr">
         <is>
           <t>75445</t>
         </is>
@@ -7145,7 +7175,7 @@
           <t>LUCATO Eleonora</t>
         </is>
       </c>
-      <c r="U117" t="inlineStr">
+      <c r="X117" t="inlineStr">
         <is>
           <t>35222</t>
         </is>
@@ -7203,7 +7233,7 @@
           <t>HAMER-EVANS Megan</t>
         </is>
       </c>
-      <c r="U118" t="inlineStr">
+      <c r="X118" t="inlineStr">
         <is>
           <t>55138</t>
         </is>
@@ -7261,7 +7291,7 @@
           <t>MASLEN Amber</t>
         </is>
       </c>
-      <c r="U119" t="inlineStr">
+      <c r="X119" t="inlineStr">
         <is>
           <t>53074</t>
         </is>
@@ -7319,7 +7349,7 @@
           <t>STANOVSKA Sona</t>
         </is>
       </c>
-      <c r="U120" t="inlineStr">
+      <c r="X120" t="inlineStr">
         <is>
           <t>51647</t>
         </is>
@@ -7377,7 +7407,7 @@
           <t>TAKESHITA Yuriko</t>
         </is>
       </c>
-      <c r="U121" t="inlineStr">
+      <c r="X121" t="inlineStr">
         <is>
           <t>36487</t>
         </is>
@@ -7435,7 +7465,7 @@
           <t>NOVAK Ajda</t>
         </is>
       </c>
-      <c r="U122" t="inlineStr">
+      <c r="X122" t="inlineStr">
         <is>
           <t>39079</t>
         </is>
@@ -7493,7 +7523,7 @@
           <t>NEVARILOVA Kristina</t>
         </is>
       </c>
-      <c r="U123" t="inlineStr">
+      <c r="X123" t="inlineStr">
         <is>
           <t>35467</t>
         </is>
@@ -7551,7 +7581,7 @@
           <t>US Viktoriia</t>
         </is>
       </c>
-      <c r="U124" t="inlineStr">
+      <c r="X124" t="inlineStr">
         <is>
           <t>35528</t>
         </is>
@@ -7609,7 +7639,7 @@
           <t>LEITNER Lisa</t>
         </is>
       </c>
-      <c r="U125" t="inlineStr">
+      <c r="X125" t="inlineStr">
         <is>
           <t>35305</t>
         </is>
@@ -7879,7 +7909,7 @@
           <t>MICOZZI Elena</t>
         </is>
       </c>
-      <c r="U130" t="inlineStr">
+      <c r="X130" t="inlineStr">
         <is>
           <t>84644</t>
         </is>
@@ -7937,7 +7967,7 @@
           <t>HOCEVAR Eva Alina</t>
         </is>
       </c>
-      <c r="U131" t="inlineStr">
+      <c r="X131" t="inlineStr">
         <is>
           <t>75533</t>
         </is>
@@ -7995,7 +8025,7 @@
           <t>CHUNG Yu-Han</t>
         </is>
       </c>
-      <c r="U132" t="inlineStr">
+      <c r="X132" t="inlineStr">
         <is>
           <t>51895</t>
         </is>
@@ -8053,7 +8083,7 @@
           <t>MARX Alena</t>
         </is>
       </c>
-      <c r="U133" t="inlineStr">
+      <c r="X133" t="inlineStr">
         <is>
           <t>68844</t>
         </is>
@@ -8111,7 +8141,7 @@
           <t>MILLER Ellis</t>
         </is>
       </c>
-      <c r="U134" t="inlineStr">
+      <c r="X134" t="inlineStr">
         <is>
           <t>75828</t>
         </is>
@@ -8169,7 +8199,7 @@
           <t>JANSSEN Fanchon</t>
         </is>
       </c>
-      <c r="U135" t="inlineStr">
+      <c r="X135" t="inlineStr">
         <is>
           <t>71963</t>
         </is>
@@ -8227,7 +8257,7 @@
           <t>MISHIMA Ren</t>
         </is>
       </c>
-      <c r="U136" t="inlineStr">
+      <c r="X136" t="inlineStr">
         <is>
           <t>37757</t>
         </is>
@@ -8285,7 +8315,7 @@
           <t>HENRY Margaux</t>
         </is>
       </c>
-      <c r="U137" t="inlineStr">
+      <c r="X137" t="inlineStr">
         <is>
           <t>51995</t>
         </is>
@@ -8343,7 +8373,7 @@
           <t>OGILVIE Sophie</t>
         </is>
       </c>
-      <c r="U138" t="inlineStr">
+      <c r="X138" t="inlineStr">
         <is>
           <t>53134</t>
         </is>
@@ -8401,7 +8431,7 @@
           <t>NOVAK Lea</t>
         </is>
       </c>
-      <c r="U139" t="inlineStr">
+      <c r="X139" t="inlineStr">
         <is>
           <t>60323</t>
         </is>
@@ -8459,7 +8489,7 @@
           <t>SATO Ayano</t>
         </is>
       </c>
-      <c r="U140" t="inlineStr">
+      <c r="X140" t="inlineStr">
         <is>
           <t>60374</t>
         </is>
@@ -8517,7 +8547,7 @@
           <t>BERTONCELLI Marta</t>
         </is>
       </c>
-      <c r="U141" t="inlineStr">
+      <c r="X141" t="inlineStr">
         <is>
           <t>71982</t>
         </is>
@@ -8575,7 +8605,7 @@
           <t>WALL Demelza</t>
         </is>
       </c>
-      <c r="U142" t="inlineStr">
+      <c r="X142" t="inlineStr">
         <is>
           <t>60107</t>
         </is>
@@ -8633,7 +8663,7 @@
           <t>DELASSUS Marjorie</t>
         </is>
       </c>
-      <c r="U143" t="inlineStr">
+      <c r="X143" t="inlineStr">
         <is>
           <t>71964</t>
         </is>
@@ -8691,7 +8721,7 @@
           <t>GLEJTEKOVA Simona</t>
         </is>
       </c>
-      <c r="U144" t="inlineStr">
+      <c r="X144" t="inlineStr">
         <is>
           <t>55166</t>
         </is>
@@ -8749,7 +8779,7 @@
           <t>DOBROTVORSKA Viktoriia</t>
         </is>
       </c>
-      <c r="U145" t="inlineStr">
+      <c r="X145" t="inlineStr">
         <is>
           <t>35526</t>
         </is>
@@ -8807,7 +8837,7 @@
           <t>RIHOVA Eva</t>
         </is>
       </c>
-      <c r="U146" t="inlineStr">
+      <c r="X146" t="inlineStr">
         <is>
           <t>51791</t>
         </is>
@@ -8865,7 +8895,7 @@
           <t>US Viktoriia</t>
         </is>
       </c>
-      <c r="U147" t="inlineStr">
+      <c r="X147" t="inlineStr">
         <is>
           <t>35528</t>
         </is>
@@ -8923,7 +8953,7 @@
           <t>MATULKOVA Jana</t>
         </is>
       </c>
-      <c r="U148" t="inlineStr">
+      <c r="X148" t="inlineStr">
         <is>
           <t>37274</t>
         </is>
@@ -8981,7 +9011,7 @@
           <t>BIZJAK Nina</t>
         </is>
       </c>
-      <c r="U149" t="inlineStr">
+      <c r="X149" t="inlineStr">
         <is>
           <t>39984</t>
         </is>
@@ -9039,7 +9069,7 @@
           <t>DONNELLY Sage</t>
         </is>
       </c>
-      <c r="U150" t="inlineStr">
+      <c r="X150" t="inlineStr">
         <is>
           <t>60119</t>
         </is>
@@ -9097,7 +9127,7 @@
           <t>STANOVSKA Sona</t>
         </is>
       </c>
-      <c r="U151" t="inlineStr">
+      <c r="X151" t="inlineStr">
         <is>
           <t>51647</t>
         </is>
@@ -9155,7 +9185,7 @@
           <t>SKACHOVA Monika</t>
         </is>
       </c>
-      <c r="U152" t="inlineStr">
+      <c r="X152" t="inlineStr">
         <is>
           <t>53078</t>
         </is>
@@ -9213,7 +9243,7 @@
           <t>HERZOG Andrea</t>
         </is>
       </c>
-      <c r="U153" t="inlineStr">
+      <c r="X153" t="inlineStr">
         <is>
           <t>55099</t>
         </is>
@@ -9271,7 +9301,7 @@
           <t>STOECKLIN Lena</t>
         </is>
       </c>
-      <c r="U154" t="inlineStr">
+      <c r="X154" t="inlineStr">
         <is>
           <t>35822</t>
         </is>
@@ -9329,7 +9359,7 @@
           <t>WOLFFHARDT Viktoria</t>
         </is>
       </c>
-      <c r="U155" t="inlineStr">
+      <c r="X155" t="inlineStr">
         <is>
           <t>35303</t>
         </is>
@@ -9387,7 +9417,7 @@
           <t>LAWRENCE Rosalyn</t>
         </is>
       </c>
-      <c r="U156" t="inlineStr">
+      <c r="X156" t="inlineStr">
         <is>
           <t>36531</t>
         </is>
@@ -9445,7 +9475,7 @@
           <t>WERATSCHNIG Nadine</t>
         </is>
       </c>
-      <c r="U157" t="inlineStr">
+      <c r="X157" t="inlineStr">
         <is>
           <t>41613</t>
         </is>
@@ -9503,7 +9533,7 @@
           <t>FISEROVA Tereza</t>
         </is>
       </c>
-      <c r="U158" t="inlineStr">
+      <c r="X158" t="inlineStr">
         <is>
           <t>42016</t>
         </is>
@@ -9561,7 +9591,7 @@
           <t>FOX Jessica</t>
         </is>
       </c>
-      <c r="U159" t="inlineStr">
+      <c r="X159" t="inlineStr">
         <is>
           <t>36526</t>
         </is>
@@ -9619,7 +9649,7 @@
           <t>DELAHAYE Vincent</t>
         </is>
       </c>
-      <c r="U160" t="inlineStr">
+      <c r="X160" t="inlineStr">
         <is>
           <t>85203</t>
         </is>
@@ -9677,7 +9707,7 @@
           <t>ANSELL Sean</t>
         </is>
       </c>
-      <c r="U161" t="inlineStr">
+      <c r="X161" t="inlineStr">
         <is>
           <t>70054</t>
         </is>
@@ -9735,7 +9765,7 @@
           <t>SANTOS Luca</t>
         </is>
       </c>
-      <c r="U162" t="inlineStr">
+      <c r="X162" t="inlineStr">
         <is>
           <t>69115</t>
         </is>
@@ -9793,7 +9823,7 @@
           <t>DELASSUS Anatole</t>
         </is>
       </c>
-      <c r="U163" t="inlineStr">
+      <c r="X163" t="inlineStr">
         <is>
           <t>84109</t>
         </is>
@@ -9904,7 +9934,7 @@
           <t>SWETNAM Huw</t>
         </is>
       </c>
-      <c r="U165" t="inlineStr">
+      <c r="X165" t="inlineStr">
         <is>
           <t>35652</t>
         </is>
@@ -9962,7 +9992,7 @@
           <t>HAYWARD Ben</t>
         </is>
       </c>
-      <c r="U166" t="inlineStr">
+      <c r="X166" t="inlineStr">
         <is>
           <t>35539</t>
         </is>
@@ -10020,7 +10050,7 @@
           <t>POLACZYK Rafal</t>
         </is>
       </c>
-      <c r="U167" t="inlineStr">
+      <c r="X167" t="inlineStr">
         <is>
           <t>35083</t>
         </is>
@@ -10078,7 +10108,7 @@
           <t>LONCAR Mihael</t>
         </is>
       </c>
-      <c r="U168" t="inlineStr">
+      <c r="X168" t="inlineStr">
         <is>
           <t>53744</t>
         </is>
@@ -10136,7 +10166,7 @@
           <t>FARRELL Oisin</t>
         </is>
       </c>
-      <c r="U169" t="inlineStr">
+      <c r="X169" t="inlineStr">
         <is>
           <t>37916</t>
         </is>
@@ -10194,7 +10224,7 @@
           <t>RACZ Koppany</t>
         </is>
       </c>
-      <c r="U170" t="inlineStr">
+      <c r="X170" t="inlineStr">
         <is>
           <t>69570</t>
         </is>
@@ -10252,7 +10282,7 @@
           <t>ECHEVERRIA OLGUIN Andraz</t>
         </is>
       </c>
-      <c r="U171" t="inlineStr">
+      <c r="X171" t="inlineStr">
         <is>
           <t>41646</t>
         </is>
@@ -10310,7 +10340,7 @@
           <t>HENDRICK Noel</t>
         </is>
       </c>
-      <c r="U172" t="inlineStr">
+      <c r="X172" t="inlineStr">
         <is>
           <t>43003</t>
         </is>
@@ -10368,7 +10398,7 @@
           <t>SOUDI Mathis</t>
         </is>
       </c>
-      <c r="U173" t="inlineStr">
+      <c r="X173" t="inlineStr">
         <is>
           <t>69447</t>
         </is>
@@ -10426,7 +10456,7 @@
           <t>STANOVSKY Samuel</t>
         </is>
       </c>
-      <c r="U174" t="inlineStr">
+      <c r="X174" t="inlineStr">
         <is>
           <t>84121</t>
         </is>
@@ -10484,7 +10514,7 @@
           <t>JOSEPH Joshua</t>
         </is>
       </c>
-      <c r="U175" t="inlineStr">
+      <c r="X175" t="inlineStr">
         <is>
           <t>69141</t>
         </is>
@@ -10542,7 +10572,7 @@
           <t>WESTFALL Tyler</t>
         </is>
       </c>
-      <c r="U176" t="inlineStr">
+      <c r="X176" t="inlineStr">
         <is>
           <t>51919</t>
         </is>
@@ -10600,7 +10630,7 @@
           <t>KORPES Ren</t>
         </is>
       </c>
-      <c r="U177" t="inlineStr">
+      <c r="X177" t="inlineStr">
         <is>
           <t>39941</t>
         </is>
@@ -10658,7 +10688,7 @@
           <t>LEE EDWARDS Ciaran</t>
         </is>
       </c>
-      <c r="U178" t="inlineStr">
+      <c r="X178" t="inlineStr">
         <is>
           <t>35614</t>
         </is>
@@ -10716,7 +10746,7 @@
           <t>THOMPSON Angus</t>
         </is>
       </c>
-      <c r="U179" t="inlineStr">
+      <c r="X179" t="inlineStr">
         <is>
           <t>44814</t>
         </is>
@@ -10774,7 +10804,7 @@
           <t>STAHL Lukas</t>
         </is>
       </c>
-      <c r="U180" t="inlineStr">
+      <c r="X180" t="inlineStr">
         <is>
           <t>55115</t>
         </is>
@@ -10832,7 +10862,7 @@
           <t>MARX Dimitri</t>
         </is>
       </c>
-      <c r="U181" t="inlineStr">
+      <c r="X181" t="inlineStr">
         <is>
           <t>60326</t>
         </is>
@@ -10890,7 +10920,7 @@
           <t>WAHLEN Fredrik</t>
         </is>
       </c>
-      <c r="U182" t="inlineStr">
+      <c r="X182" t="inlineStr">
         <is>
           <t>35102</t>
         </is>
@@ -10948,7 +10978,7 @@
           <t>CHIARELLO Gelindo</t>
         </is>
       </c>
-      <c r="U183" t="inlineStr">
+      <c r="X183" t="inlineStr">
         <is>
           <t>39956</t>
         </is>
@@ -11006,7 +11036,7 @@
           <t>YOSHIDA Taku</t>
         </is>
       </c>
-      <c r="U184" t="inlineStr">
+      <c r="X184" t="inlineStr">
         <is>
           <t>41611</t>
         </is>
@@ -11064,7 +11094,7 @@
           <t>PESTOV Ruslan</t>
         </is>
       </c>
-      <c r="U185" t="inlineStr">
+      <c r="X185" t="inlineStr">
         <is>
           <t>36138</t>
         </is>
@@ -11122,7 +11152,7 @@
           <t>STANOVSKY Martin</t>
         </is>
       </c>
-      <c r="U186" t="inlineStr">
+      <c r="X186" t="inlineStr">
         <is>
           <t>68782</t>
         </is>
@@ -11180,7 +11210,7 @@
           <t>QUEMENEUR Malo</t>
         </is>
       </c>
-      <c r="U187" t="inlineStr">
+      <c r="X187" t="inlineStr">
         <is>
           <t>60403</t>
         </is>
@@ -11238,7 +11268,7 @@
           <t>POPE Benjamin</t>
         </is>
       </c>
-      <c r="U188" t="inlineStr">
+      <c r="X188" t="inlineStr">
         <is>
           <t>51753</t>
         </is>
@@ -11296,7 +11326,7 @@
           <t>DE DIONIGI Christian</t>
         </is>
       </c>
-      <c r="U189" t="inlineStr">
+      <c r="X189" t="inlineStr">
         <is>
           <t>43188</t>
         </is>
@@ -11354,7 +11384,7 @@
           <t>TESTEN Niko</t>
         </is>
       </c>
-      <c r="U190" t="inlineStr">
+      <c r="X190" t="inlineStr">
         <is>
           <t>39980</t>
         </is>
@@ -11412,7 +11442,7 @@
           <t>YAZAWA Kazuki</t>
         </is>
       </c>
-      <c r="U191" t="inlineStr">
+      <c r="X191" t="inlineStr">
         <is>
           <t>36482</t>
         </is>
@@ -11470,7 +11500,7 @@
           <t>HOLMER Erik</t>
         </is>
       </c>
-      <c r="U192" t="inlineStr">
+      <c r="X192" t="inlineStr">
         <is>
           <t>35104</t>
         </is>
@@ -11528,7 +11558,7 @@
           <t>GILBERT Callum</t>
         </is>
       </c>
-      <c r="U193" t="inlineStr">
+      <c r="X193" t="inlineStr">
         <is>
           <t>42090</t>
         </is>
@@ -11586,7 +11616,7 @@
           <t>WEGER Jakob</t>
         </is>
       </c>
-      <c r="U194" t="inlineStr">
+      <c r="X194" t="inlineStr">
         <is>
           <t>54909</t>
         </is>
@@ -11644,7 +11674,7 @@
           <t>WEGER Matthias</t>
         </is>
       </c>
-      <c r="U195" t="inlineStr">
+      <c r="X195" t="inlineStr">
         <is>
           <t>68837</t>
         </is>
@@ -11702,7 +11732,7 @@
           <t>JAKSE Zan</t>
         </is>
       </c>
-      <c r="U196" t="inlineStr">
+      <c r="X196" t="inlineStr">
         <is>
           <t>44340</t>
         </is>
@@ -11760,7 +11790,7 @@
           <t>TSVIET Igor</t>
         </is>
       </c>
-      <c r="U197" t="inlineStr">
+      <c r="X197" t="inlineStr">
         <is>
           <t>35527</t>
         </is>
@@ -11818,7 +11848,7 @@
           <t>LEITNER Mario</t>
         </is>
       </c>
-      <c r="U198" t="inlineStr">
+      <c r="X198" t="inlineStr">
         <is>
           <t>35546</t>
         </is>
@@ -11876,7 +11906,7 @@
           <t>MALEK Andrej</t>
         </is>
       </c>
-      <c r="U199" t="inlineStr">
+      <c r="X199" t="inlineStr">
         <is>
           <t>39246</t>
         </is>
@@ -11934,7 +11964,7 @@
           <t>SRABOTNIK Martin</t>
         </is>
       </c>
-      <c r="U200" t="inlineStr">
+      <c r="X200" t="inlineStr">
         <is>
           <t>39080</t>
         </is>
@@ -11992,7 +12022,7 @@
           <t>HALCIN Martin</t>
         </is>
       </c>
-      <c r="U201" t="inlineStr">
+      <c r="X201" t="inlineStr">
         <is>
           <t>35355</t>
         </is>
@@ -12050,7 +12080,7 @@
           <t>OSCHMAUTZ Felix</t>
         </is>
       </c>
-      <c r="U202" t="inlineStr">
+      <c r="X202" t="inlineStr">
         <is>
           <t>51856</t>
         </is>
@@ -12108,7 +12138,7 @@
           <t>PASIUT Michal</t>
         </is>
       </c>
-      <c r="U203" t="inlineStr">
+      <c r="X203" t="inlineStr">
         <is>
           <t>35095</t>
         </is>
@@ -12166,7 +12196,7 @@
           <t>HILGERT Lubos</t>
         </is>
       </c>
-      <c r="U204" t="inlineStr">
+      <c r="X204" t="inlineStr">
         <is>
           <t>35032</t>
         </is>
@@ -12224,7 +12254,7 @@
           <t>OHRSTROM Isak</t>
         </is>
       </c>
-      <c r="U205" t="inlineStr">
+      <c r="X205" t="inlineStr">
         <is>
           <t>35101</t>
         </is>
@@ -12282,7 +12312,7 @@
           <t>IVALDI Zeno</t>
         </is>
       </c>
-      <c r="U206" t="inlineStr">
+      <c r="X206" t="inlineStr">
         <is>
           <t>35480</t>
         </is>
@@ -12340,7 +12370,7 @@
           <t>MAXEINER Tim</t>
         </is>
       </c>
-      <c r="U207" t="inlineStr">
+      <c r="X207" t="inlineStr">
         <is>
           <t>35117</t>
         </is>
@@ -12398,7 +12428,7 @@
           <t>ADACHI Kazuya</t>
         </is>
       </c>
-      <c r="U208" t="inlineStr">
+      <c r="X208" t="inlineStr">
         <is>
           <t>36646</t>
         </is>
@@ -12456,7 +12486,7 @@
           <t>POLACZYK Mateusz</t>
         </is>
       </c>
-      <c r="U209" t="inlineStr">
+      <c r="X209" t="inlineStr">
         <is>
           <t>35072</t>
         </is>
@@ -12514,7 +12544,7 @@
           <t>BIAZIZZO Mathieu</t>
         </is>
       </c>
-      <c r="U210" t="inlineStr">
+      <c r="X210" t="inlineStr">
         <is>
           <t>35484</t>
         </is>
@@ -12572,7 +12602,7 @@
           <t>SMOLEN Michal</t>
         </is>
       </c>
-      <c r="U211" t="inlineStr">
+      <c r="X211" t="inlineStr">
         <is>
           <t>36397</t>
         </is>
@@ -12630,7 +12660,7 @@
           <t>POPIELA Dariusz</t>
         </is>
       </c>
-      <c r="U212" t="inlineStr">
+      <c r="X212" t="inlineStr">
         <is>
           <t>35096</t>
         </is>
@@ -12688,7 +12718,7 @@
           <t>TUNKA Ondrej</t>
         </is>
       </c>
-      <c r="U213" t="inlineStr">
+      <c r="X213" t="inlineStr">
         <is>
           <t>35947</t>
         </is>
@@ -12746,7 +12776,7 @@
           <t>GRIGAR Jakub</t>
         </is>
       </c>
-      <c r="U214" t="inlineStr">
+      <c r="X214" t="inlineStr">
         <is>
           <t>37284</t>
         </is>
@@ -12804,7 +12834,7 @@
           <t>AIGNER Hannes</t>
         </is>
       </c>
-      <c r="U215" t="inlineStr">
+      <c r="X215" t="inlineStr">
         <is>
           <t>35115</t>
         </is>
@@ -12862,7 +12892,7 @@
           <t>SCHUBERT Sebastian</t>
         </is>
       </c>
-      <c r="U216" t="inlineStr">
+      <c r="X216" t="inlineStr">
         <is>
           <t>35114</t>
         </is>
@@ -12920,7 +12950,7 @@
           <t>PRSKAVEC Jiri</t>
         </is>
       </c>
-      <c r="U217" t="inlineStr">
+      <c r="X217" t="inlineStr">
         <is>
           <t>35033</t>
         </is>
@@ -12978,7 +13008,7 @@
           <t>PRINDIS Vit</t>
         </is>
       </c>
-      <c r="U218" t="inlineStr">
+      <c r="X218" t="inlineStr">
         <is>
           <t>35065</t>
         </is>
@@ -13036,7 +13066,7 @@
           <t>KAUZER Peter</t>
         </is>
       </c>
-      <c r="U219" t="inlineStr">
+      <c r="X219" t="inlineStr">
         <is>
           <t>35589</t>
         </is>
@@ -13094,7 +13124,7 @@
           <t>MICOZZI Elena</t>
         </is>
       </c>
-      <c r="U220" t="inlineStr">
+      <c r="X220" t="inlineStr">
         <is>
           <t>84644</t>
         </is>
@@ -13152,7 +13182,7 @@
           <t>CHUNG Yu-Han</t>
         </is>
       </c>
-      <c r="U221" t="inlineStr">
+      <c r="X221" t="inlineStr">
         <is>
           <t>51895</t>
         </is>
@@ -13210,7 +13240,7 @@
           <t>MARX Alena</t>
         </is>
       </c>
-      <c r="U222" t="inlineStr">
+      <c r="X222" t="inlineStr">
         <is>
           <t>68844</t>
         </is>
@@ -13268,7 +13298,7 @@
           <t>MISHIMA Ren</t>
         </is>
       </c>
-      <c r="U223" t="inlineStr">
+      <c r="X223" t="inlineStr">
         <is>
           <t>37757</t>
         </is>
@@ -13326,7 +13356,7 @@
           <t>OGILVIE Sophie</t>
         </is>
       </c>
-      <c r="U224" t="inlineStr">
+      <c r="X224" t="inlineStr">
         <is>
           <t>53134</t>
         </is>
@@ -13384,7 +13414,7 @@
           <t>SATO Ayano</t>
         </is>
       </c>
-      <c r="U225" t="inlineStr">
+      <c r="X225" t="inlineStr">
         <is>
           <t>60374</t>
         </is>
@@ -13442,7 +13472,7 @@
           <t>BIZJAK Nina</t>
         </is>
       </c>
-      <c r="U226" t="inlineStr">
+      <c r="X226" t="inlineStr">
         <is>
           <t>39984</t>
         </is>
@@ -13500,7 +13530,7 @@
           <t>DONNELLY Sage</t>
         </is>
       </c>
-      <c r="U227" t="inlineStr">
+      <c r="X227" t="inlineStr">
         <is>
           <t>60119</t>
         </is>
@@ -13558,7 +13588,7 @@
           <t>WERATSCHNIG Nadine</t>
         </is>
       </c>
-      <c r="U228" t="inlineStr">
+      <c r="X228" t="inlineStr">
         <is>
           <t>41613</t>
         </is>
@@ -13616,7 +13646,7 @@
           <t>FISEROVA Tereza</t>
         </is>
       </c>
-      <c r="U229" t="inlineStr">
+      <c r="X229" t="inlineStr">
         <is>
           <t>42016</t>
         </is>
@@ -13674,7 +13704,7 @@
           <t>ANSELL Sean</t>
         </is>
       </c>
-      <c r="U230" t="inlineStr">
+      <c r="X230" t="inlineStr">
         <is>
           <t>70054</t>
         </is>
@@ -13732,7 +13762,7 @@
           <t>SANTOS Luca</t>
         </is>
       </c>
-      <c r="U231" t="inlineStr">
+      <c r="X231" t="inlineStr">
         <is>
           <t>69115</t>
         </is>
@@ -13790,7 +13820,7 @@
           <t>DELASSUS Anatole</t>
         </is>
       </c>
-      <c r="U232" t="inlineStr">
+      <c r="X232" t="inlineStr">
         <is>
           <t>84109</t>
         </is>
@@ -13848,7 +13878,7 @@
           <t>SWETNAM Huw</t>
         </is>
       </c>
-      <c r="U233" t="inlineStr">
+      <c r="X233" t="inlineStr">
         <is>
           <t>35652</t>
         </is>
@@ -13906,7 +13936,7 @@
           <t>POLACZYK Rafal</t>
         </is>
       </c>
-      <c r="U234" t="inlineStr">
+      <c r="X234" t="inlineStr">
         <is>
           <t>35083</t>
         </is>
@@ -13964,7 +13994,7 @@
           <t>LONCAR Mihael</t>
         </is>
       </c>
-      <c r="U235" t="inlineStr">
+      <c r="X235" t="inlineStr">
         <is>
           <t>53744</t>
         </is>
@@ -14022,7 +14052,7 @@
           <t>FARRELL Oisin</t>
         </is>
       </c>
-      <c r="U236" t="inlineStr">
+      <c r="X236" t="inlineStr">
         <is>
           <t>37916</t>
         </is>
@@ -14080,7 +14110,7 @@
           <t>RACZ Koppany</t>
         </is>
       </c>
-      <c r="U237" t="inlineStr">
+      <c r="X237" t="inlineStr">
         <is>
           <t>69570</t>
         </is>
@@ -14138,7 +14168,7 @@
           <t>ECHEVERRIA OLGUIN Andraz</t>
         </is>
       </c>
-      <c r="U238" t="inlineStr">
+      <c r="X238" t="inlineStr">
         <is>
           <t>41646</t>
         </is>
@@ -14196,7 +14226,7 @@
           <t>HENDRICK Noel</t>
         </is>
       </c>
-      <c r="U239" t="inlineStr">
+      <c r="X239" t="inlineStr">
         <is>
           <t>43003</t>
         </is>
@@ -14254,7 +14284,7 @@
           <t>STANOVSKY Samuel</t>
         </is>
       </c>
-      <c r="U240" t="inlineStr">
+      <c r="X240" t="inlineStr">
         <is>
           <t>84121</t>
         </is>
@@ -14312,7 +14342,7 @@
           <t>JOSEPH Joshua</t>
         </is>
       </c>
-      <c r="U241" t="inlineStr">
+      <c r="X241" t="inlineStr">
         <is>
           <t>69141</t>
         </is>
@@ -14370,7 +14400,7 @@
           <t>WESTFALL Tyler</t>
         </is>
       </c>
-      <c r="U242" t="inlineStr">
+      <c r="X242" t="inlineStr">
         <is>
           <t>51919</t>
         </is>
@@ -14428,7 +14458,7 @@
           <t>KORPES Ren</t>
         </is>
       </c>
-      <c r="U243" t="inlineStr">
+      <c r="X243" t="inlineStr">
         <is>
           <t>39941</t>
         </is>
@@ -14486,7 +14516,7 @@
           <t>LEE EDWARDS Ciaran</t>
         </is>
       </c>
-      <c r="U244" t="inlineStr">
+      <c r="X244" t="inlineStr">
         <is>
           <t>35614</t>
         </is>
@@ -14544,7 +14574,7 @@
           <t>MARX Dimitri</t>
         </is>
       </c>
-      <c r="U245" t="inlineStr">
+      <c r="X245" t="inlineStr">
         <is>
           <t>60326</t>
         </is>
@@ -14602,7 +14632,7 @@
           <t>WAHLEN Fredrik</t>
         </is>
       </c>
-      <c r="U246" t="inlineStr">
+      <c r="X246" t="inlineStr">
         <is>
           <t>35102</t>
         </is>
@@ -14660,7 +14690,7 @@
           <t>CHIARELLO Gelindo</t>
         </is>
       </c>
-      <c r="U247" t="inlineStr">
+      <c r="X247" t="inlineStr">
         <is>
           <t>39956</t>
         </is>
@@ -14718,7 +14748,7 @@
           <t>YOSHIDA Taku</t>
         </is>
       </c>
-      <c r="U248" t="inlineStr">
+      <c r="X248" t="inlineStr">
         <is>
           <t>41611</t>
         </is>
@@ -14776,7 +14806,7 @@
           <t>PESTOV Ruslan</t>
         </is>
       </c>
-      <c r="U249" t="inlineStr">
+      <c r="X249" t="inlineStr">
         <is>
           <t>36138</t>
         </is>
@@ -14834,7 +14864,7 @@
           <t>STANOVSKY Martin</t>
         </is>
       </c>
-      <c r="U250" t="inlineStr">
+      <c r="X250" t="inlineStr">
         <is>
           <t>68782</t>
         </is>
@@ -14892,7 +14922,7 @@
           <t>QUEMENEUR Malo</t>
         </is>
       </c>
-      <c r="U251" t="inlineStr">
+      <c r="X251" t="inlineStr">
         <is>
           <t>60403</t>
         </is>
@@ -14950,7 +14980,7 @@
           <t>POPE Benjamin</t>
         </is>
       </c>
-      <c r="U252" t="inlineStr">
+      <c r="X252" t="inlineStr">
         <is>
           <t>51753</t>
         </is>
@@ -15008,7 +15038,7 @@
           <t>DE DIONIGI Christian</t>
         </is>
       </c>
-      <c r="U253" t="inlineStr">
+      <c r="X253" t="inlineStr">
         <is>
           <t>43188</t>
         </is>
@@ -15066,7 +15096,7 @@
           <t>GILBERT Callum</t>
         </is>
       </c>
-      <c r="U254" t="inlineStr">
+      <c r="X254" t="inlineStr">
         <is>
           <t>42090</t>
         </is>
@@ -15124,7 +15154,7 @@
           <t>WEGER Jakob</t>
         </is>
       </c>
-      <c r="U255" t="inlineStr">
+      <c r="X255" t="inlineStr">
         <is>
           <t>54909</t>
         </is>
@@ -15182,7 +15212,7 @@
           <t>WEGER Matthias</t>
         </is>
       </c>
-      <c r="U256" t="inlineStr">
+      <c r="X256" t="inlineStr">
         <is>
           <t>68837</t>
         </is>
@@ -15240,7 +15270,7 @@
           <t>HILGERT Lubos</t>
         </is>
       </c>
-      <c r="U257" t="inlineStr">
+      <c r="X257" t="inlineStr">
         <is>
           <t>35032</t>
         </is>
@@ -15298,7 +15328,7 @@
           <t>SMOLEN Michal</t>
         </is>
       </c>
-      <c r="U258" t="inlineStr">
+      <c r="X258" t="inlineStr">
         <is>
           <t>36397</t>
         </is>
@@ -15356,7 +15386,7 @@
           <t>GRIGAR Jakub</t>
         </is>
       </c>
-      <c r="U259" t="inlineStr">
+      <c r="X259" t="inlineStr">
         <is>
           <t>37284</t>
         </is>
@@ -15573,7 +15603,7 @@
           <t>LOKKEN Zachary</t>
         </is>
       </c>
-      <c r="U263" t="inlineStr">
+      <c r="X263" t="inlineStr">
         <is>
           <t>35069</t>
         </is>
@@ -15631,7 +15661,7 @@
           <t>LOWTHER Steven</t>
         </is>
       </c>
-      <c r="U264" t="inlineStr">
+      <c r="X264" t="inlineStr">
         <is>
           <t>44811</t>
         </is>
@@ -15689,7 +15719,7 @@
           <t>CECCON Paolo</t>
         </is>
       </c>
-      <c r="U265" t="inlineStr">
+      <c r="X265" t="inlineStr">
         <is>
           <t>39903</t>
         </is>
@@ -15747,7 +15777,7 @@
           <t>TRUMMER Timo</t>
         </is>
       </c>
-      <c r="U266" t="inlineStr">
+      <c r="X266" t="inlineStr">
         <is>
           <t>41599</t>
         </is>
@@ -15805,7 +15835,7 @@
           <t>JANE Michal</t>
         </is>
       </c>
-      <c r="U267" t="inlineStr">
+      <c r="X267" t="inlineStr">
         <is>
           <t>35059</t>
         </is>
@@ -15916,7 +15946,7 @@
           <t>ABBOTT Thomas</t>
         </is>
       </c>
-      <c r="U269" t="inlineStr">
+      <c r="X269" t="inlineStr">
         <is>
           <t>36514</t>
         </is>
@@ -15974,7 +16004,7 @@
           <t>RAK Tomas</t>
         </is>
       </c>
-      <c r="U270" t="inlineStr">
+      <c r="X270" t="inlineStr">
         <is>
           <t>35056</t>
         </is>
@@ -16032,7 +16062,7 @@
           <t>MARINIC Matija</t>
         </is>
       </c>
-      <c r="U271" t="inlineStr">
+      <c r="X271" t="inlineStr">
         <is>
           <t>35595</t>
         </is>
@@ -16090,7 +16120,7 @@
           <t>GARGAUD CHANUT Denis</t>
         </is>
       </c>
-      <c r="U272" t="inlineStr">
+      <c r="X272" t="inlineStr">
         <is>
           <t>35177</t>
         </is>
@@ -16148,7 +16178,7 @@
           <t>BOURHIS Yves</t>
         </is>
       </c>
-      <c r="U273" t="inlineStr">
+      <c r="X273" t="inlineStr">
         <is>
           <t>63237</t>
         </is>
@@ -16206,7 +16236,7 @@
           <t>SZTUBA Igor</t>
         </is>
       </c>
-      <c r="U274" t="inlineStr">
+      <c r="X274" t="inlineStr">
         <is>
           <t>35087</t>
         </is>
@@ -16317,7 +16347,7 @@
           <t>ROHAN Lukas</t>
         </is>
       </c>
-      <c r="U276" t="inlineStr">
+      <c r="X276" t="inlineStr">
         <is>
           <t>36114</t>
         </is>
@@ -16375,7 +16405,7 @@
           <t>SZTUBA Kacper</t>
         </is>
       </c>
-      <c r="U277" t="inlineStr">
+      <c r="X277" t="inlineStr">
         <is>
           <t>53636</t>
         </is>
@@ -16433,7 +16463,7 @@
           <t>MIRGORODSKY Marko</t>
         </is>
       </c>
-      <c r="U278" t="inlineStr">
+      <c r="X278" t="inlineStr">
         <is>
           <t>42019</t>
         </is>
@@ -16491,7 +16521,7 @@
           <t>GESTIN Nicolas</t>
         </is>
       </c>
-      <c r="U279" t="inlineStr">
+      <c r="X279" t="inlineStr">
         <is>
           <t>71961</t>
         </is>
@@ -16549,7 +16579,7 @@
           <t>HEDWIG Grzegorz</t>
         </is>
       </c>
-      <c r="U280" t="inlineStr">
+      <c r="X280" t="inlineStr">
         <is>
           <t>35465</t>
         </is>
@@ -16607,7 +16637,7 @@
           <t>MARTIKAN Michal</t>
         </is>
       </c>
-      <c r="U281" t="inlineStr">
+      <c r="X281" t="inlineStr">
         <is>
           <t>35365</t>
         </is>
@@ -16665,7 +16695,7 @@
           <t>TILLARD Pierre-Antoine</t>
         </is>
       </c>
-      <c r="U282" t="inlineStr">
+      <c r="X282" t="inlineStr">
         <is>
           <t>35413</t>
         </is>
@@ -16723,7 +16753,7 @@
           <t>TASIADIS Sideris</t>
         </is>
       </c>
-      <c r="U283" t="inlineStr">
+      <c r="X283" t="inlineStr">
         <is>
           <t>35135</t>
         </is>
@@ -16781,7 +16811,7 @@
           <t>EICHFELD Casey</t>
         </is>
       </c>
-      <c r="U284" t="inlineStr">
+      <c r="X284" t="inlineStr">
         <is>
           <t>35067</t>
         </is>
@@ -16839,7 +16869,7 @@
           <t>ANTON Franz</t>
         </is>
       </c>
-      <c r="U285" t="inlineStr">
+      <c r="X285" t="inlineStr">
         <is>
           <t>35137</t>
         </is>
@@ -16897,7 +16927,7 @@
           <t>JOLY Cedric</t>
         </is>
       </c>
-      <c r="U286" t="inlineStr">
+      <c r="X286" t="inlineStr">
         <is>
           <t>35681</t>
         </is>
@@ -16955,7 +16985,7 @@
           <t>BENUS Matej</t>
         </is>
       </c>
-      <c r="U287" t="inlineStr">
+      <c r="X287" t="inlineStr">
         <is>
           <t>35353</t>
         </is>
@@ -17013,7 +17043,7 @@
           <t>LENARCIC Jure</t>
         </is>
       </c>
-      <c r="U288" t="inlineStr">
+      <c r="X288" t="inlineStr">
         <is>
           <t>36259</t>
         </is>
@@ -17071,7 +17101,7 @@
           <t>SAVSEK Benjamin</t>
         </is>
       </c>
-      <c r="U289" t="inlineStr">
+      <c r="X289" t="inlineStr">
         <is>
           <t>36218</t>
         </is>
@@ -17129,7 +17159,7 @@
           <t>BERCIC Anze</t>
         </is>
       </c>
-      <c r="U290" t="inlineStr">
+      <c r="X290" t="inlineStr">
         <is>
           <t>36253</t>
         </is>
@@ -17187,7 +17217,7 @@
           <t>BOZIC Luka</t>
         </is>
       </c>
-      <c r="U291" t="inlineStr">
+      <c r="X291" t="inlineStr">
         <is>
           <t>36269</t>
         </is>
@@ -17245,7 +17275,7 @@
           <t>SLAFKOVSKY Alexander</t>
         </is>
       </c>
-      <c r="U292" t="inlineStr">
+      <c r="X292" t="inlineStr">
         <is>
           <t>35129</t>
         </is>
@@ -17303,7 +17333,7 @@
           <t>TAKESHITA Yuriko</t>
         </is>
       </c>
-      <c r="U293" t="inlineStr">
+      <c r="X293" t="inlineStr">
         <is>
           <t>36487</t>
         </is>
@@ -17361,7 +17391,7 @@
           <t>RIHOVA Eva</t>
         </is>
       </c>
-      <c r="U294" t="inlineStr">
+      <c r="X294" t="inlineStr">
         <is>
           <t>51791</t>
         </is>
@@ -17419,7 +17449,7 @@
           <t>OGILVIE Sophie</t>
         </is>
       </c>
-      <c r="U295" t="inlineStr">
+      <c r="X295" t="inlineStr">
         <is>
           <t>53134</t>
         </is>
@@ -17477,7 +17507,7 @@
           <t>MASLEN Amber</t>
         </is>
       </c>
-      <c r="U296" t="inlineStr">
+      <c r="X296" t="inlineStr">
         <is>
           <t>53074</t>
         </is>
@@ -17535,7 +17565,7 @@
           <t>DELASSUS Marjorie</t>
         </is>
       </c>
-      <c r="U297" t="inlineStr">
+      <c r="X297" t="inlineStr">
         <is>
           <t>71964</t>
         </is>
@@ -17593,7 +17623,7 @@
           <t>LEAVER Lois</t>
         </is>
       </c>
-      <c r="U298" t="inlineStr">
+      <c r="X298" t="inlineStr">
         <is>
           <t>83842</t>
         </is>
@@ -17651,7 +17681,7 @@
           <t>STANOVSKA Sona</t>
         </is>
       </c>
-      <c r="U299" t="inlineStr">
+      <c r="X299" t="inlineStr">
         <is>
           <t>51647</t>
         </is>
@@ -17709,7 +17739,7 @@
           <t>SRIBAR Ria</t>
         </is>
       </c>
-      <c r="U300" t="inlineStr">
+      <c r="X300" t="inlineStr">
         <is>
           <t>75645</t>
         </is>
@@ -17767,7 +17797,7 @@
           <t>HAMER-EVANS Megan</t>
         </is>
       </c>
-      <c r="U301" t="inlineStr">
+      <c r="X301" t="inlineStr">
         <is>
           <t>55138</t>
         </is>
@@ -17825,7 +17855,7 @@
           <t>LEITNER Lisa</t>
         </is>
       </c>
-      <c r="U302" t="inlineStr">
+      <c r="X302" t="inlineStr">
         <is>
           <t>35305</t>
         </is>
@@ -17883,7 +17913,7 @@
           <t>OSCHMAUTZ Antonia</t>
         </is>
       </c>
-      <c r="U303" t="inlineStr">
+      <c r="X303" t="inlineStr">
         <is>
           <t>68839</t>
         </is>
@@ -17941,7 +17971,7 @@
           <t>NEE Ashley</t>
         </is>
       </c>
-      <c r="U304" t="inlineStr">
+      <c r="X304" t="inlineStr">
         <is>
           <t>36363</t>
         </is>
@@ -17999,7 +18029,7 @@
           <t>LAWRENCE Rosalyn</t>
         </is>
       </c>
-      <c r="U305" t="inlineStr">
+      <c r="X305" t="inlineStr">
         <is>
           <t>36531</t>
         </is>
@@ -18057,7 +18087,7 @@
           <t>WEGMAN Martina</t>
         </is>
       </c>
-      <c r="U306" t="inlineStr">
+      <c r="X306" t="inlineStr">
         <is>
           <t>35345</t>
         </is>
@@ -18115,7 +18145,7 @@
           <t>FABER Anna</t>
         </is>
       </c>
-      <c r="U307" t="inlineStr">
+      <c r="X307" t="inlineStr">
         <is>
           <t>39059</t>
         </is>
@@ -18173,7 +18203,7 @@
           <t>YAZAWA Aki</t>
         </is>
       </c>
-      <c r="U308" t="inlineStr">
+      <c r="X308" t="inlineStr">
         <is>
           <t>36486</t>
         </is>
@@ -18231,7 +18261,7 @@
           <t>LAFONT Marie-Zelia</t>
         </is>
       </c>
-      <c r="U309" t="inlineStr">
+      <c r="X309" t="inlineStr">
         <is>
           <t>35374</t>
         </is>
@@ -18289,7 +18319,7 @@
           <t>TERCELJ Eva</t>
         </is>
       </c>
-      <c r="U310" t="inlineStr">
+      <c r="X310" t="inlineStr">
         <is>
           <t>36263</t>
         </is>
@@ -18347,7 +18377,7 @@
           <t>PRIGENT Camille</t>
         </is>
       </c>
-      <c r="U311" t="inlineStr">
+      <c r="X311" t="inlineStr">
         <is>
           <t>41566</t>
         </is>
@@ -18405,7 +18435,7 @@
           <t>KUDEJOVA Katerina</t>
         </is>
       </c>
-      <c r="U312" t="inlineStr">
+      <c r="X312" t="inlineStr">
         <is>
           <t>35034</t>
         </is>
@@ -18463,7 +18493,7 @@
           <t>VOJTOVA Veronika</t>
         </is>
       </c>
-      <c r="U313" t="inlineStr">
+      <c r="X313" t="inlineStr">
         <is>
           <t>35945</t>
         </is>
@@ -18521,7 +18551,7 @@
           <t>ZWOLINSKA Klaudia</t>
         </is>
       </c>
-      <c r="U314" t="inlineStr">
+      <c r="X314" t="inlineStr">
         <is>
           <t>42027</t>
         </is>
@@ -18579,7 +18609,7 @@
           <t>HILGERTOVA Amalie</t>
         </is>
       </c>
-      <c r="U315" t="inlineStr">
+      <c r="X315" t="inlineStr">
         <is>
           <t>36113</t>
         </is>
@@ -18637,7 +18667,7 @@
           <t>FOX Jessica</t>
         </is>
       </c>
-      <c r="U316" t="inlineStr">
+      <c r="X316" t="inlineStr">
         <is>
           <t>36526</t>
         </is>
@@ -18695,7 +18725,7 @@
           <t>SCHORNBERG Jasmin</t>
         </is>
       </c>
-      <c r="U317" t="inlineStr">
+      <c r="X317" t="inlineStr">
         <is>
           <t>35206</t>
         </is>
@@ -18753,7 +18783,7 @@
           <t>WOLFFHARDT Viktoria</t>
         </is>
       </c>
-      <c r="U318" t="inlineStr">
+      <c r="X318" t="inlineStr">
         <is>
           <t>35303</t>
         </is>
@@ -18811,7 +18841,7 @@
           <t>HORN Stefanie</t>
         </is>
       </c>
-      <c r="U319" t="inlineStr">
+      <c r="X319" t="inlineStr">
         <is>
           <t>38417</t>
         </is>
@@ -18869,7 +18899,7 @@
           <t>KRAGELJ Ursa</t>
         </is>
       </c>
-      <c r="U320" t="inlineStr">
+      <c r="X320" t="inlineStr">
         <is>
           <t>36264</t>
         </is>
@@ -18927,7 +18957,7 @@
           <t>KUHNLE Corinna</t>
         </is>
       </c>
-      <c r="U321" t="inlineStr">
+      <c r="X321" t="inlineStr">
         <is>
           <t>35282</t>
         </is>
@@ -18985,7 +19015,7 @@
           <t>FUNK Ricarda</t>
         </is>
       </c>
-      <c r="U322" t="inlineStr">
+      <c r="X322" t="inlineStr">
         <is>
           <t>35122</t>
         </is>
@@ -19053,7 +19083,7 @@
           <t>ANTON Franz</t>
         </is>
       </c>
-      <c r="U323" t="inlineStr">
+      <c r="X323" t="inlineStr">
         <is>
           <t>35137</t>
         </is>
@@ -19121,7 +19151,7 @@
           <t>BOZIC Luka</t>
         </is>
       </c>
-      <c r="U324" t="inlineStr">
+      <c r="X324" t="inlineStr">
         <is>
           <t>36269</t>
         </is>
@@ -19189,7 +19219,7 @@
           <t>BERCIC Anze</t>
         </is>
       </c>
-      <c r="U325" t="inlineStr">
+      <c r="X325" t="inlineStr">
         <is>
           <t>36253</t>
         </is>
@@ -19257,7 +19287,7 @@
           <t>MARTIKAN Michal</t>
         </is>
       </c>
-      <c r="U326" t="inlineStr">
+      <c r="X326" t="inlineStr">
         <is>
           <t>35365</t>
         </is>
@@ -19325,7 +19355,7 @@
           <t>HEDWIG Grzegorz</t>
         </is>
       </c>
-      <c r="U327" t="inlineStr">
+      <c r="X327" t="inlineStr">
         <is>
           <t>35465</t>
         </is>
@@ -19393,7 +19423,7 @@
           <t>TASIADIS Sideris</t>
         </is>
       </c>
-      <c r="U328" t="inlineStr">
+      <c r="X328" t="inlineStr">
         <is>
           <t>35135</t>
         </is>
@@ -19461,7 +19491,7 @@
           <t>LENARCIC Jure</t>
         </is>
       </c>
-      <c r="U329" t="inlineStr">
+      <c r="X329" t="inlineStr">
         <is>
           <t>36259</t>
         </is>
@@ -19529,7 +19559,7 @@
           <t>GESTIN Nicolas</t>
         </is>
       </c>
-      <c r="U330" t="inlineStr">
+      <c r="X330" t="inlineStr">
         <is>
           <t>71961</t>
         </is>
@@ -19597,7 +19627,7 @@
           <t>SAVSEK Benjamin</t>
         </is>
       </c>
-      <c r="U331" t="inlineStr">
+      <c r="X331" t="inlineStr">
         <is>
           <t>36218</t>
         </is>
@@ -19665,7 +19695,7 @@
           <t>SLAFKOVSKY Alexander</t>
         </is>
       </c>
-      <c r="U332" t="inlineStr">
+      <c r="X332" t="inlineStr">
         <is>
           <t>35129</t>
         </is>
@@ -19733,7 +19763,7 @@
           <t>LEITNER Lisa</t>
         </is>
       </c>
-      <c r="U333" t="inlineStr">
+      <c r="X333" t="inlineStr">
         <is>
           <t>35305</t>
         </is>
@@ -19801,7 +19831,7 @@
           <t>LAWRENCE Rosalyn</t>
         </is>
       </c>
-      <c r="U334" t="inlineStr">
+      <c r="X334" t="inlineStr">
         <is>
           <t>36531</t>
         </is>
@@ -19869,7 +19899,7 @@
           <t>KUDEJOVA Katerina</t>
         </is>
       </c>
-      <c r="U335" t="inlineStr">
+      <c r="X335" t="inlineStr">
         <is>
           <t>35034</t>
         </is>
@@ -19937,7 +19967,7 @@
           <t>TERCELJ Eva</t>
         </is>
       </c>
-      <c r="U336" t="inlineStr">
+      <c r="X336" t="inlineStr">
         <is>
           <t>36263</t>
         </is>
@@ -20005,7 +20035,7 @@
           <t>SCHORNBERG Jasmin</t>
         </is>
       </c>
-      <c r="U337" t="inlineStr">
+      <c r="X337" t="inlineStr">
         <is>
           <t>35206</t>
         </is>
@@ -20073,7 +20103,7 @@
           <t>FUNK Ricarda</t>
         </is>
       </c>
-      <c r="U338" t="inlineStr">
+      <c r="X338" t="inlineStr">
         <is>
           <t>35122</t>
         </is>
@@ -20141,7 +20171,7 @@
           <t>WOLFFHARDT Viktoria</t>
         </is>
       </c>
-      <c r="U339" t="inlineStr">
+      <c r="X339" t="inlineStr">
         <is>
           <t>35303</t>
         </is>
@@ -20209,7 +20239,7 @@
           <t>KRAGELJ Ursa</t>
         </is>
       </c>
-      <c r="U340" t="inlineStr">
+      <c r="X340" t="inlineStr">
         <is>
           <t>36264</t>
         </is>
@@ -20277,7 +20307,7 @@
           <t>KUHNLE Corinna</t>
         </is>
       </c>
-      <c r="U341" t="inlineStr">
+      <c r="X341" t="inlineStr">
         <is>
           <t>35282</t>
         </is>
@@ -20345,7 +20375,7 @@
           <t>FOX Jessica</t>
         </is>
       </c>
-      <c r="U342" t="inlineStr">
+      <c r="X342" t="inlineStr">
         <is>
           <t>36526</t>
         </is>
@@ -20408,12 +20438,12 @@
           <t>MRUZEK Vojtech</t>
         </is>
       </c>
-      <c r="U343" t="inlineStr">
+      <c r="X343" t="inlineStr">
         <is>
           <t>37274</t>
         </is>
       </c>
-      <c r="V343" t="inlineStr">
+      <c r="Y343" t="inlineStr">
         <is>
           <t>42012</t>
         </is>
@@ -20476,12 +20506,12 @@
           <t>HENRY Margaux</t>
         </is>
       </c>
-      <c r="U344" t="inlineStr">
+      <c r="X344" t="inlineStr">
         <is>
           <t>35671</t>
         </is>
       </c>
-      <c r="V344" t="inlineStr">
+      <c r="Y344" t="inlineStr">
         <is>
           <t>51995</t>
         </is>
@@ -20544,12 +20574,12 @@
           <t>MASEK Jan</t>
         </is>
       </c>
-      <c r="U345" t="inlineStr">
+      <c r="X345" t="inlineStr">
         <is>
           <t>35945</t>
         </is>
       </c>
-      <c r="V345" t="inlineStr">
+      <c r="Y345" t="inlineStr">
         <is>
           <t>36013</t>
         </is>
@@ -20612,7 +20642,12 @@
           <t>JANE Jakub</t>
         </is>
       </c>
-      <c r="V346" t="inlineStr">
+      <c r="X346" t="inlineStr">
+        <is>
+          <t>42016</t>
+        </is>
+      </c>
+      <c r="Y346" t="inlineStr">
         <is>
           <t>35061</t>
         </is>
@@ -20685,12 +20720,12 @@
           <t>HENRY Margaux</t>
         </is>
       </c>
-      <c r="U347" t="inlineStr">
+      <c r="X347" t="inlineStr">
         <is>
           <t>35671</t>
         </is>
       </c>
-      <c r="V347" t="inlineStr">
+      <c r="Y347" t="inlineStr">
         <is>
           <t>51995</t>
         </is>
@@ -20763,12 +20798,12 @@
           <t>MASEK Jan</t>
         </is>
       </c>
-      <c r="U348" t="inlineStr">
+      <c r="X348" t="inlineStr">
         <is>
           <t>35945</t>
         </is>
       </c>
-      <c r="V348" t="inlineStr">
+      <c r="Y348" t="inlineStr">
         <is>
           <t>36013</t>
         </is>
@@ -20841,12 +20876,12 @@
           <t>MRUZEK Vojtech</t>
         </is>
       </c>
-      <c r="U349" t="inlineStr">
+      <c r="X349" t="inlineStr">
         <is>
           <t>37274</t>
         </is>
       </c>
-      <c r="V349" t="inlineStr">
+      <c r="Y349" t="inlineStr">
         <is>
           <t>42012</t>
         </is>
@@ -20919,7 +20954,12 @@
           <t>JANE Jakub</t>
         </is>
       </c>
-      <c r="V350" t="inlineStr">
+      <c r="X350" t="inlineStr">
+        <is>
+          <t>42016</t>
+        </is>
+      </c>
+      <c r="Y350" t="inlineStr">
         <is>
           <t>35061</t>
         </is>
@@ -20982,7 +21022,7 @@
           <t>CHAPPELL Etienne</t>
         </is>
       </c>
-      <c r="U351" t="inlineStr">
+      <c r="X351" t="inlineStr">
         <is>
           <t>75833</t>
         </is>
@@ -21045,7 +21085,7 @@
           <t>MUTTON Zack</t>
         </is>
       </c>
-      <c r="U352" t="inlineStr">
+      <c r="X352" t="inlineStr">
         <is>
           <t>51827</t>
         </is>
@@ -21108,7 +21148,7 @@
           <t>SMOLEN Michal</t>
         </is>
       </c>
-      <c r="U353" t="inlineStr">
+      <c r="X353" t="inlineStr">
         <is>
           <t>36397</t>
         </is>
@@ -21171,7 +21211,7 @@
           <t>ANSELL Sean</t>
         </is>
       </c>
-      <c r="U354" t="inlineStr">
+      <c r="X354" t="inlineStr">
         <is>
           <t>70054</t>
         </is>
@@ -21234,7 +21274,7 @@
           <t>KORPES Ren</t>
         </is>
       </c>
-      <c r="U355" t="inlineStr">
+      <c r="X355" t="inlineStr">
         <is>
           <t>39941</t>
         </is>
@@ -21297,7 +21337,7 @@
           <t>STANOVSKY Samuel</t>
         </is>
       </c>
-      <c r="U356" t="inlineStr">
+      <c r="X356" t="inlineStr">
         <is>
           <t>84121</t>
         </is>
@@ -21360,7 +21400,7 @@
           <t>WESTFALL Tyler</t>
         </is>
       </c>
-      <c r="U357" t="inlineStr">
+      <c r="X357" t="inlineStr">
         <is>
           <t>51919</t>
         </is>
@@ -21423,7 +21463,7 @@
           <t>FARRELL Oisin</t>
         </is>
       </c>
-      <c r="U358" t="inlineStr">
+      <c r="X358" t="inlineStr">
         <is>
           <t>37916</t>
         </is>
@@ -21486,7 +21526,7 @@
           <t>HAYWARD Ben</t>
         </is>
       </c>
-      <c r="U359" t="inlineStr">
+      <c r="X359" t="inlineStr">
         <is>
           <t>35539</t>
         </is>
@@ -21549,7 +21589,7 @@
           <t>PETEK Marko</t>
         </is>
       </c>
-      <c r="U360" t="inlineStr">
+      <c r="X360" t="inlineStr">
         <is>
           <t>83907</t>
         </is>
@@ -21612,7 +21652,7 @@
           <t>POLACZYK Rafal</t>
         </is>
       </c>
-      <c r="U361" t="inlineStr">
+      <c r="X361" t="inlineStr">
         <is>
           <t>35083</t>
         </is>
@@ -21675,7 +21715,7 @@
           <t>KANCLER Tine</t>
         </is>
       </c>
-      <c r="U362" t="inlineStr">
+      <c r="X362" t="inlineStr">
         <is>
           <t>51813</t>
         </is>
@@ -21738,7 +21778,7 @@
           <t>STANOVSKY Martin</t>
         </is>
       </c>
-      <c r="U363" t="inlineStr">
+      <c r="X363" t="inlineStr">
         <is>
           <t>68782</t>
         </is>
@@ -21801,7 +21841,7 @@
           <t>WAHLEN Fredrik</t>
         </is>
       </c>
-      <c r="U364" t="inlineStr">
+      <c r="X364" t="inlineStr">
         <is>
           <t>35102</t>
         </is>
@@ -21864,7 +21904,7 @@
           <t>DOMANJKO Helena</t>
         </is>
       </c>
-      <c r="U365" t="inlineStr">
+      <c r="X365" t="inlineStr">
         <is>
           <t>83895</t>
         </is>
@@ -21927,7 +21967,7 @@
           <t>WEGMAN Martina</t>
         </is>
       </c>
-      <c r="U366" t="inlineStr">
+      <c r="X366" t="inlineStr">
         <is>
           <t>35345</t>
         </is>
@@ -21990,7 +22030,7 @@
           <t>DONNELLY Sage</t>
         </is>
       </c>
-      <c r="U367" t="inlineStr">
+      <c r="X367" t="inlineStr">
         <is>
           <t>60119</t>
         </is>
@@ -22053,7 +22093,7 @@
           <t>NEE Ashley</t>
         </is>
       </c>
-      <c r="U368" t="inlineStr">
+      <c r="X368" t="inlineStr">
         <is>
           <t>36363</t>
         </is>

</xml_diff>